<commit_message>
implemented promotions generator and its working
</commit_message>
<xml_diff>
--- a/generator/output/master/stores.xlsx
+++ b/generator/output/master/stores.xlsx
@@ -485,7 +485,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Naivas Karen Branch</t>
+          <t>Naivas Nyali Branch</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -499,28 +499,28 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>1068</v>
+        <v>1007</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Nairobi</t>
+          <t>Mombasa</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Nairobi</t>
+          <t>Coast</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Karen</t>
+          <t>Nyali</t>
         </is>
       </c>
       <c r="I2" s="1" t="n">
-        <v>42953</v>
+        <v>42094</v>
       </c>
       <c r="J2" s="1" t="n">
-        <v>45211</v>
+        <v>44041</v>
       </c>
       <c r="K2" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
complete project setup and working correctly
</commit_message>
<xml_diff>
--- a/generator/output/master/stores.xlsx
+++ b/generator/output/master/stores.xlsx
@@ -485,7 +485,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Tuskys Naivasha Branch</t>
+          <t>Tuskys Nyeri Town Branch</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -495,32 +495,32 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Hypermarket</t>
+          <t>Express</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>8563</v>
+        <v>1012</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Nakuru</t>
+          <t>Nyeri</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Rift Valley</t>
+          <t>Central</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Naivasha</t>
+          <t>Nyeri Town</t>
         </is>
       </c>
       <c r="I2" s="1" t="n">
-        <v>42506</v>
+        <v>42744</v>
       </c>
       <c r="J2" s="1" t="n">
-        <v>44746</v>
+        <v>45128</v>
       </c>
       <c r="K2" t="b">
         <v>1</v>
@@ -534,7 +534,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Quickmart Kitale Branch</t>
+          <t>Quickmart Embu Town Branch</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -544,32 +544,32 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Express</t>
+          <t>Supermarket</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>1692</v>
+        <v>4718</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Trans Nzoia</t>
+          <t>Embu</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Rift Valley</t>
+          <t>Eastern</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Kitale</t>
+          <t>Embu Town</t>
         </is>
       </c>
       <c r="I3" s="1" t="n">
-        <v>43521</v>
+        <v>43169</v>
       </c>
       <c r="J3" s="1" t="n">
-        <v>44188</v>
+        <v>45555</v>
       </c>
       <c r="K3" t="b">
         <v>1</v>
@@ -583,42 +583,42 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Eastmatt Kakamega Town Branch</t>
+          <t>Cleanshelf Makutano Branch</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Eastmatt</t>
+          <t>Cleanshelf</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Hypermarket</t>
+          <t>Express</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>8191</v>
+        <v>1176</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Kakamega</t>
+          <t>Meru</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Western</t>
+          <t>Eastern</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Kakamega Town</t>
+          <t>Makutano</t>
         </is>
       </c>
       <c r="I4" s="1" t="n">
-        <v>42452</v>
+        <v>43567</v>
       </c>
       <c r="J4" s="1" t="n">
-        <v>44784</v>
+        <v>45761</v>
       </c>
       <c r="K4" t="b">
         <v>1</v>
@@ -632,42 +632,42 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Naivas Maua Branch</t>
+          <t>Tuskys Gilgil Branch</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Naivas</t>
+          <t>Tuskys</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Express</t>
+          <t>Hypermarket</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>1733</v>
+        <v>8138</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Meru</t>
+          <t>Nakuru</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Eastern</t>
+          <t>Rift Valley</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Maua</t>
+          <t>Gilgil</t>
         </is>
       </c>
       <c r="I5" s="1" t="n">
-        <v>43335</v>
+        <v>42033</v>
       </c>
       <c r="J5" s="1" t="n">
-        <v>45550</v>
+        <v>44905</v>
       </c>
       <c r="K5" t="b">
         <v>1</v>
@@ -681,7 +681,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Carrefour Diani Branch</t>
+          <t>Carrefour Maua Branch</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -691,32 +691,32 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Express</t>
+          <t>Hypermarket</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>1284</v>
+        <v>8123</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Kwale</t>
+          <t>Meru</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Coast</t>
+          <t>Eastern</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Diani</t>
+          <t>Maua</t>
         </is>
       </c>
       <c r="I6" s="1" t="n">
-        <v>43662</v>
+        <v>43621</v>
       </c>
       <c r="J6" s="1" t="n">
-        <v>43858</v>
+        <v>45462</v>
       </c>
       <c r="K6" t="b">
         <v>1</v>
@@ -730,12 +730,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Quickmart Kikuyu Branch</t>
+          <t>Chandarana Ruaka Branch</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Quickmart</t>
+          <t>Chandarana</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -744,28 +744,28 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>1348</v>
+        <v>1513</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Kiambu</t>
+          <t>Nairobi</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Central</t>
+          <t>Nairobi</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Kikuyu</t>
+          <t>Ruaka</t>
         </is>
       </c>
       <c r="I7" s="1" t="n">
-        <v>42574</v>
+        <v>43576</v>
       </c>
       <c r="J7" s="1" t="n">
-        <v>44468</v>
+        <v>45533</v>
       </c>
       <c r="K7" t="b">
         <v>1</v>
@@ -779,12 +779,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Carrefour Kisumu City Branch</t>
+          <t>Eastmatt Ruiru Branch</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Carrefour</t>
+          <t>Eastmatt</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -793,28 +793,28 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>1344</v>
+        <v>1084</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Kisumu</t>
+          <t>Kiambu</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Nyanza</t>
+          <t>Central</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Kisumu City</t>
+          <t>Ruiru</t>
         </is>
       </c>
       <c r="I8" s="1" t="n">
-        <v>42214</v>
+        <v>43316</v>
       </c>
       <c r="J8" s="1" t="n">
-        <v>44211</v>
+        <v>44457</v>
       </c>
       <c r="K8" t="b">
         <v>1</v>
@@ -828,12 +828,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Eastmatt Bungoma Town Branch</t>
+          <t>Chandarana Athi River Branch</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Eastmatt</t>
+          <t>Chandarana</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -842,28 +842,28 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>9735</v>
+        <v>8161</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Bungoma</t>
+          <t>Machakos</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Western</t>
+          <t>Eastern</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Bungoma Town</t>
+          <t>Athi River</t>
         </is>
       </c>
       <c r="I9" s="1" t="n">
-        <v>42709</v>
+        <v>43052</v>
       </c>
       <c r="J9" s="1" t="n">
-        <v>44915</v>
+        <v>44664</v>
       </c>
       <c r="K9" t="b">
         <v>1</v>
@@ -877,12 +877,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Naivas Nakuru Town Branch</t>
+          <t>Quickmart Ruiru Branch</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Naivas</t>
+          <t>Quickmart</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -891,28 +891,28 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>1549</v>
+        <v>1400</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Nakuru</t>
+          <t>Kiambu</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Rift Valley</t>
+          <t>Central</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Nakuru Town</t>
+          <t>Ruiru</t>
         </is>
       </c>
       <c r="I10" s="1" t="n">
-        <v>42260</v>
+        <v>43206</v>
       </c>
       <c r="J10" s="1" t="n">
-        <v>45382</v>
+        <v>44102</v>
       </c>
       <c r="K10" t="b">
         <v>1</v>
@@ -926,12 +926,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Tuskys Meru Town Branch</t>
+          <t>Chandarana Embu Town Branch</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Tuskys</t>
+          <t>Chandarana</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -940,11 +940,11 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>1849</v>
+        <v>1747</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Meru</t>
+          <t>Embu</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -954,14 +954,14 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Meru Town</t>
+          <t>Embu Town</t>
         </is>
       </c>
       <c r="I11" s="1" t="n">
-        <v>43292</v>
+        <v>43738</v>
       </c>
       <c r="J11" s="1" t="n">
-        <v>45313</v>
+        <v>44809</v>
       </c>
       <c r="K11" t="b">
         <v>1</v>
@@ -975,25 +975,25 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Carrefour Nakuru Town Branch</t>
+          <t>Naivas Nanyuki Branch</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Carrefour</t>
+          <t>Naivas</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Express</t>
+          <t>Supermarket</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>1046</v>
+        <v>4893</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Nakuru</t>
+          <t>Laikipia</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1003,14 +1003,14 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Nakuru Town</t>
+          <t>Nanyuki</t>
         </is>
       </c>
       <c r="I12" s="1" t="n">
-        <v>43359</v>
+        <v>42894</v>
       </c>
       <c r="J12" s="1" t="n">
-        <v>44765</v>
+        <v>44307</v>
       </c>
       <c r="K12" t="b">
         <v>1</v>
@@ -1024,12 +1024,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Chandarana Kilifi Town Branch</t>
+          <t>Magunas Kakamega Town Branch</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Chandarana</t>
+          <t>Magunas</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1038,28 +1038,28 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>1875</v>
+        <v>1056</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Kilifi</t>
+          <t>Kakamega</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Coast</t>
+          <t>Western</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Kilifi Town</t>
+          <t>Kakamega Town</t>
         </is>
       </c>
       <c r="I13" s="1" t="n">
-        <v>42481</v>
+        <v>42638</v>
       </c>
       <c r="J13" s="1" t="n">
-        <v>44245</v>
+        <v>44551</v>
       </c>
       <c r="K13" t="b">
         <v>1</v>
@@ -1073,42 +1073,42 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Eastmatt Murang'a Town Branch</t>
+          <t>Tuskys Mombasa CBD Branch</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Eastmatt</t>
+          <t>Tuskys</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Supermarket</t>
+          <t>Hypermarket</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>4301</v>
+        <v>8281</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Murang'a</t>
+          <t>Mombasa</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Central</t>
+          <t>Coast</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Murang'a Town</t>
+          <t>Mombasa CBD</t>
         </is>
       </c>
       <c r="I14" s="1" t="n">
-        <v>43713</v>
+        <v>43441</v>
       </c>
       <c r="J14" s="1" t="n">
-        <v>45326</v>
+        <v>43878</v>
       </c>
       <c r="K14" t="b">
         <v>1</v>
@@ -1122,7 +1122,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Quickmart Nakuru Town Branch</t>
+          <t>Quickmart Kakamega Town Branch</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1132,32 +1132,32 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Supermarket</t>
+          <t>Express</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>3429</v>
+        <v>1355</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Nakuru</t>
+          <t>Kakamega</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Rift Valley</t>
+          <t>Western</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Nakuru Town</t>
+          <t>Kakamega Town</t>
         </is>
       </c>
       <c r="I15" s="1" t="n">
-        <v>43377</v>
+        <v>43076</v>
       </c>
       <c r="J15" s="1" t="n">
-        <v>44925</v>
+        <v>45950</v>
       </c>
       <c r="K15" t="b">
         <v>1</v>
@@ -1171,42 +1171,42 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Tuskys Kasarani Branch</t>
+          <t>Chandarana Nyali Branch</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Tuskys</t>
+          <t>Chandarana</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Express</t>
+          <t>Supermarket</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>1175</v>
+        <v>3259</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Nairobi</t>
+          <t>Mombasa</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Nairobi</t>
+          <t>Coast</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Kasarani</t>
+          <t>Nyali</t>
         </is>
       </c>
       <c r="I16" s="1" t="n">
-        <v>43098</v>
+        <v>43540</v>
       </c>
       <c r="J16" s="1" t="n">
-        <v>44834</v>
+        <v>44932</v>
       </c>
       <c r="K16" t="b">
         <v>1</v>
@@ -1220,12 +1220,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Quickmart Makutano Branch</t>
+          <t>Tuskys Kakamega Town Branch</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Quickmart</t>
+          <t>Tuskys</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1234,28 +1234,28 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>1276</v>
+        <v>1030</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Meru</t>
+          <t>Kakamega</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Eastern</t>
+          <t>Western</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Makutano</t>
+          <t>Kakamega Town</t>
         </is>
       </c>
       <c r="I17" s="1" t="n">
-        <v>43315</v>
+        <v>42691</v>
       </c>
       <c r="J17" s="1" t="n">
-        <v>44731</v>
+        <v>45590</v>
       </c>
       <c r="K17" t="b">
         <v>1</v>
@@ -1269,12 +1269,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Cleanshelf Gilgil Branch</t>
+          <t>Chandarana Gilgil Branch</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Cleanshelf</t>
+          <t>Chandarana</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1283,7 +1283,7 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>1794</v>
+        <v>1269</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -1301,10 +1301,10 @@
         </is>
       </c>
       <c r="I18" s="1" t="n">
-        <v>42119</v>
+        <v>43463</v>
       </c>
       <c r="J18" s="1" t="n">
-        <v>44770</v>
+        <v>44147</v>
       </c>
       <c r="K18" t="b">
         <v>1</v>
@@ -1318,12 +1318,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Naivas Nanyuki Branch</t>
+          <t>Magunas Nanyuki Branch</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Naivas</t>
+          <t>Magunas</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1332,7 +1332,7 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>1410</v>
+        <v>1368</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -1350,10 +1350,10 @@
         </is>
       </c>
       <c r="I19" s="1" t="n">
-        <v>42553</v>
+        <v>42118</v>
       </c>
       <c r="J19" s="1" t="n">
-        <v>44103</v>
+        <v>45878</v>
       </c>
       <c r="K19" t="b">
         <v>1</v>
@@ -1367,42 +1367,42 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Carrefour Eldoret Branch</t>
+          <t>Quickmart Nyeri Town Branch</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Carrefour</t>
+          <t>Quickmart</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Express</t>
+          <t>Supermarket</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>1580</v>
+        <v>3522</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Uasin Gishu</t>
+          <t>Nyeri</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Rift Valley</t>
+          <t>Central</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Eldoret</t>
+          <t>Nyeri Town</t>
         </is>
       </c>
       <c r="I20" s="1" t="n">
-        <v>43799</v>
+        <v>43588</v>
       </c>
       <c r="J20" s="1" t="n">
-        <v>45120</v>
+        <v>44253</v>
       </c>
       <c r="K20" t="b">
         <v>1</v>
@@ -1416,42 +1416,42 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Carrefour Meru Town Branch</t>
+          <t>Tuskys Bungoma Town Branch</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Carrefour</t>
+          <t>Tuskys</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Express</t>
+          <t>Supermarket</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>1405</v>
+        <v>4042</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Meru</t>
+          <t>Bungoma</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Eastern</t>
+          <t>Western</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Meru Town</t>
+          <t>Bungoma Town</t>
         </is>
       </c>
       <c r="I21" s="1" t="n">
-        <v>43816</v>
+        <v>42010</v>
       </c>
       <c r="J21" s="1" t="n">
-        <v>45711</v>
+        <v>44012</v>
       </c>
       <c r="K21" t="b">
         <v>1</v>
@@ -1465,12 +1465,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Quickmart Athi River Branch</t>
+          <t>Naivas Murang'a Town Branch</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Quickmart</t>
+          <t>Naivas</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1479,28 +1479,28 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>3505</v>
+        <v>3966</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Machakos</t>
+          <t>Murang'a</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Eastern</t>
+          <t>Central</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Athi River</t>
+          <t>Murang'a Town</t>
         </is>
       </c>
       <c r="I22" s="1" t="n">
-        <v>43530</v>
+        <v>42750</v>
       </c>
       <c r="J22" s="1" t="n">
-        <v>44908</v>
+        <v>45400</v>
       </c>
       <c r="K22" t="b">
         <v>1</v>
@@ -1514,42 +1514,42 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Eastmatt Athi River Branch</t>
+          <t>Quickmart Kilimani Branch</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Eastmatt</t>
+          <t>Quickmart</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Express</t>
+          <t>Supermarket</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>1408</v>
+        <v>4966</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Machakos</t>
+          <t>Nairobi</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Eastern</t>
+          <t>Nairobi</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Athi River</t>
+          <t>Kilimani</t>
         </is>
       </c>
       <c r="I23" s="1" t="n">
-        <v>42746</v>
+        <v>43761</v>
       </c>
       <c r="J23" s="1" t="n">
-        <v>44730</v>
+        <v>43976</v>
       </c>
       <c r="K23" t="b">
         <v>1</v>
@@ -1563,21 +1563,21 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Quickmart Eastleigh Branch</t>
+          <t>Eastmatt Westlands Branch</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Quickmart</t>
+          <t>Eastmatt</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Express</t>
+          <t>Supermarket</t>
         </is>
       </c>
       <c r="E24" t="n">
-        <v>1093</v>
+        <v>3508</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
@@ -1591,14 +1591,14 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Eastleigh</t>
+          <t>Westlands</t>
         </is>
       </c>
       <c r="I24" s="1" t="n">
-        <v>43552</v>
+        <v>42857</v>
       </c>
       <c r="J24" s="1" t="n">
-        <v>44024</v>
+        <v>45142</v>
       </c>
       <c r="K24" t="b">
         <v>1</v>
@@ -1612,42 +1612,42 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Tuskys Kilifi Town Branch</t>
+          <t>Chandarana Meru Town Branch</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Tuskys</t>
+          <t>Chandarana</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Supermarket</t>
+          <t>Express</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>3327</v>
+        <v>1585</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Kilifi</t>
+          <t>Meru</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Coast</t>
+          <t>Eastern</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Kilifi Town</t>
+          <t>Meru Town</t>
         </is>
       </c>
       <c r="I25" s="1" t="n">
-        <v>43627</v>
+        <v>42768</v>
       </c>
       <c r="J25" s="1" t="n">
-        <v>45561</v>
+        <v>44321</v>
       </c>
       <c r="K25" t="b">
         <v>1</v>
@@ -1661,12 +1661,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Tuskys Murang'a Town Branch</t>
+          <t>Naivas Kakamega Town Branch</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Tuskys</t>
+          <t>Naivas</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1675,28 +1675,28 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>4220</v>
+        <v>4647</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Murang'a</t>
+          <t>Kakamega</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Central</t>
+          <t>Western</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Murang'a Town</t>
+          <t>Kakamega Town</t>
         </is>
       </c>
       <c r="I26" s="1" t="n">
-        <v>42963</v>
+        <v>43061</v>
       </c>
       <c r="J26" s="1" t="n">
-        <v>45999</v>
+        <v>44020</v>
       </c>
       <c r="K26" t="b">
         <v>1</v>
@@ -1710,42 +1710,42 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Chandarana Mlolongo Branch</t>
+          <t>Eastmatt Kitale Branch</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Chandarana</t>
+          <t>Eastmatt</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Express</t>
+          <t>Hypermarket</t>
         </is>
       </c>
       <c r="E27" t="n">
-        <v>1881</v>
+        <v>8952</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Machakos</t>
+          <t>Trans Nzoia</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Eastern</t>
+          <t>Rift Valley</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Mlolongo</t>
+          <t>Kitale</t>
         </is>
       </c>
       <c r="I27" s="1" t="n">
-        <v>42028</v>
+        <v>43778</v>
       </c>
       <c r="J27" s="1" t="n">
-        <v>44301</v>
+        <v>44988</v>
       </c>
       <c r="K27" t="b">
         <v>1</v>
@@ -1759,7 +1759,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Chandarana Kasarani Branch</t>
+          <t>Chandarana Kerugoya Branch</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1769,32 +1769,32 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Express</t>
+          <t>Supermarket</t>
         </is>
       </c>
       <c r="E28" t="n">
-        <v>1348</v>
+        <v>4132</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Nairobi</t>
+          <t>Kirinyaga</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Nairobi</t>
+          <t>Central</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Kasarani</t>
+          <t>Kerugoya</t>
         </is>
       </c>
       <c r="I28" s="1" t="n">
-        <v>42233</v>
+        <v>42940</v>
       </c>
       <c r="J28" s="1" t="n">
-        <v>45034</v>
+        <v>43864</v>
       </c>
       <c r="K28" t="b">
         <v>1</v>
@@ -1808,12 +1808,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Eastmatt Kitengela Branch</t>
+          <t>Cleanshelf Westlands Branch</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Eastmatt</t>
+          <t>Cleanshelf</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1822,28 +1822,28 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>3006</v>
+        <v>4154</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Kajiado</t>
+          <t>Nairobi</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Rift Valley</t>
+          <t>Nairobi</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Kitengela</t>
+          <t>Westlands</t>
         </is>
       </c>
       <c r="I29" s="1" t="n">
-        <v>43483</v>
+        <v>43611</v>
       </c>
       <c r="J29" s="1" t="n">
-        <v>44910</v>
+        <v>45076</v>
       </c>
       <c r="K29" t="b">
         <v>1</v>
@@ -1857,12 +1857,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Quickmart Naivasha Branch</t>
+          <t>Carrefour Nanyuki Branch</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Quickmart</t>
+          <t>Carrefour</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1871,11 +1871,11 @@
         </is>
       </c>
       <c r="E30" t="n">
-        <v>1108</v>
+        <v>1605</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Nakuru</t>
+          <t>Laikipia</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -1885,14 +1885,14 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Naivasha</t>
+          <t>Nanyuki</t>
         </is>
       </c>
       <c r="I30" s="1" t="n">
-        <v>43787</v>
+        <v>43015</v>
       </c>
       <c r="J30" s="1" t="n">
-        <v>45054</v>
+        <v>44632</v>
       </c>
       <c r="K30" t="b">
         <v>1</v>
@@ -1906,7 +1906,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Carrefour Kilimani Branch</t>
+          <t>Carrefour Kakamega Town Branch</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1920,28 +1920,28 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>4561</v>
+        <v>4909</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Nairobi</t>
+          <t>Kakamega</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Nairobi</t>
+          <t>Western</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Kilimani</t>
+          <t>Kakamega Town</t>
         </is>
       </c>
       <c r="I31" s="1" t="n">
-        <v>42335</v>
+        <v>42844</v>
       </c>
       <c r="J31" s="1" t="n">
-        <v>46004</v>
+        <v>43929</v>
       </c>
       <c r="K31" t="b">
         <v>1</v>
@@ -1955,12 +1955,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Naivas Machakos Town Branch</t>
+          <t>Carrefour Murang'a Town Branch</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Naivas</t>
+          <t>Carrefour</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1969,28 +1969,28 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>1500</v>
+        <v>1651</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Machakos</t>
+          <t>Murang'a</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Eastern</t>
+          <t>Central</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Machakos Town</t>
+          <t>Murang'a Town</t>
         </is>
       </c>
       <c r="I32" s="1" t="n">
-        <v>42044</v>
+        <v>43724</v>
       </c>
       <c r="J32" s="1" t="n">
-        <v>44290</v>
+        <v>43871</v>
       </c>
       <c r="K32" t="b">
         <v>1</v>
@@ -2004,7 +2004,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Cleanshelf Nanyuki Branch</t>
+          <t>Cleanshelf Thika Branch</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -2014,29 +2014,29 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Express</t>
+          <t>Hypermarket</t>
         </is>
       </c>
       <c r="E33" t="n">
-        <v>1851</v>
+        <v>9346</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Laikipia</t>
+          <t>Kiambu</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Rift Valley</t>
+          <t>Central</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Nanyuki</t>
+          <t>Thika</t>
         </is>
       </c>
       <c r="I33" s="1" t="n">
-        <v>43657</v>
+        <v>42775</v>
       </c>
       <c r="J33" s="1" t="n">
         <v>45091</v>
@@ -2053,42 +2053,42 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Carrefour Embu Town Branch</t>
+          <t>Tuskys Kiambu Town Branch</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Carrefour</t>
+          <t>Tuskys</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Hypermarket</t>
+          <t>Supermarket</t>
         </is>
       </c>
       <c r="E34" t="n">
-        <v>9798</v>
+        <v>3487</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Embu</t>
+          <t>Kiambu</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Eastern</t>
+          <t>Central</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Embu Town</t>
+          <t>Kiambu Town</t>
         </is>
       </c>
       <c r="I34" s="1" t="n">
-        <v>43166</v>
+        <v>42864</v>
       </c>
       <c r="J34" s="1" t="n">
-        <v>44154</v>
+        <v>45847</v>
       </c>
       <c r="K34" t="b">
         <v>1</v>
@@ -2102,12 +2102,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Tuskys Ruaka Branch</t>
+          <t>Naivas Gilgil Branch</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Tuskys</t>
+          <t>Naivas</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -2116,28 +2116,28 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>1835</v>
+        <v>1145</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Nairobi</t>
+          <t>Nakuru</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Nairobi</t>
+          <t>Rift Valley</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Ruaka</t>
+          <t>Gilgil</t>
         </is>
       </c>
       <c r="I35" s="1" t="n">
-        <v>42146</v>
+        <v>43462</v>
       </c>
       <c r="J35" s="1" t="n">
-        <v>46013</v>
+        <v>44978</v>
       </c>
       <c r="K35" t="b">
         <v>1</v>
@@ -2151,42 +2151,42 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Quickmart Gilgil Branch</t>
+          <t>Tuskys Kilifi Town Branch</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Quickmart</t>
+          <t>Tuskys</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Supermarket</t>
+          <t>Hypermarket</t>
         </is>
       </c>
       <c r="E36" t="n">
-        <v>3973</v>
+        <v>8474</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Nakuru</t>
+          <t>Kilifi</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Rift Valley</t>
+          <t>Coast</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Gilgil</t>
+          <t>Kilifi Town</t>
         </is>
       </c>
       <c r="I36" s="1" t="n">
-        <v>43130</v>
+        <v>43736</v>
       </c>
       <c r="J36" s="1" t="n">
-        <v>44508</v>
+        <v>45960</v>
       </c>
       <c r="K36" t="b">
         <v>1</v>
@@ -2200,12 +2200,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Chandarana Ruaka Branch</t>
+          <t>Eastmatt Kakamega Town Branch</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Chandarana</t>
+          <t>Eastmatt</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -2214,28 +2214,28 @@
         </is>
       </c>
       <c r="E37" t="n">
-        <v>1621</v>
+        <v>1381</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Nairobi</t>
+          <t>Kakamega</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Nairobi</t>
+          <t>Western</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Ruaka</t>
+          <t>Kakamega Town</t>
         </is>
       </c>
       <c r="I37" s="1" t="n">
-        <v>42871</v>
+        <v>42943</v>
       </c>
       <c r="J37" s="1" t="n">
-        <v>44699</v>
+        <v>44179</v>
       </c>
       <c r="K37" t="b">
         <v>1</v>
@@ -2249,12 +2249,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Carrefour Kikuyu Branch</t>
+          <t>Tuskys Kitale Branch</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Carrefour</t>
+          <t>Tuskys</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -2263,28 +2263,28 @@
         </is>
       </c>
       <c r="E38" t="n">
-        <v>1408</v>
+        <v>1652</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Kiambu</t>
+          <t>Trans Nzoia</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Central</t>
+          <t>Rift Valley</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Kikuyu</t>
+          <t>Kitale</t>
         </is>
       </c>
       <c r="I38" s="1" t="n">
-        <v>43380</v>
+        <v>43684</v>
       </c>
       <c r="J38" s="1" t="n">
-        <v>45361</v>
+        <v>45447</v>
       </c>
       <c r="K38" t="b">
         <v>1</v>
@@ -2298,12 +2298,12 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Magunas Kiambu Town Branch</t>
+          <t>Tuskys Naivasha Branch</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Magunas</t>
+          <t>Tuskys</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -2312,28 +2312,28 @@
         </is>
       </c>
       <c r="E39" t="n">
-        <v>1462</v>
+        <v>1063</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Kiambu</t>
+          <t>Nakuru</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Central</t>
+          <t>Rift Valley</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Kiambu Town</t>
+          <t>Naivasha</t>
         </is>
       </c>
       <c r="I39" s="1" t="n">
-        <v>42252</v>
+        <v>42895</v>
       </c>
       <c r="J39" s="1" t="n">
-        <v>44847</v>
+        <v>44367</v>
       </c>
       <c r="K39" t="b">
         <v>1</v>
@@ -2347,7 +2347,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Carrefour Ruiru Branch</t>
+          <t>Carrefour Kikuyu Branch</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2357,11 +2357,11 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Hypermarket</t>
+          <t>Supermarket</t>
         </is>
       </c>
       <c r="E40" t="n">
-        <v>8043</v>
+        <v>4742</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
@@ -2375,14 +2375,14 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>Ruiru</t>
+          <t>Kikuyu</t>
         </is>
       </c>
       <c r="I40" s="1" t="n">
-        <v>43209</v>
+        <v>42650</v>
       </c>
       <c r="J40" s="1" t="n">
-        <v>44774</v>
+        <v>45441</v>
       </c>
       <c r="K40" t="b">
         <v>1</v>
@@ -2396,42 +2396,42 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Carrefour Athi River Branch</t>
+          <t>Cleanshelf Nyali Branch</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Carrefour</t>
+          <t>Cleanshelf</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Hypermarket</t>
+          <t>Supermarket</t>
         </is>
       </c>
       <c r="E41" t="n">
-        <v>9449</v>
+        <v>3556</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Machakos</t>
+          <t>Mombasa</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Eastern</t>
+          <t>Coast</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>Athi River</t>
+          <t>Nyali</t>
         </is>
       </c>
       <c r="I41" s="1" t="n">
-        <v>43297</v>
+        <v>42483</v>
       </c>
       <c r="J41" s="1" t="n">
-        <v>44073</v>
+        <v>44137</v>
       </c>
       <c r="K41" t="b">
         <v>1</v>
@@ -2445,7 +2445,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Carrefour Nairobi CBD Branch</t>
+          <t>Carrefour Machakos Town Branch</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2455,32 +2455,32 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Hypermarket</t>
+          <t>Supermarket</t>
         </is>
       </c>
       <c r="E42" t="n">
-        <v>8064</v>
+        <v>4577</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Nairobi</t>
+          <t>Machakos</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Nairobi</t>
+          <t>Eastern</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>Nairobi CBD</t>
+          <t>Machakos Town</t>
         </is>
       </c>
       <c r="I42" s="1" t="n">
-        <v>43765</v>
+        <v>43202</v>
       </c>
       <c r="J42" s="1" t="n">
-        <v>45185</v>
+        <v>44278</v>
       </c>
       <c r="K42" t="b">
         <v>1</v>
@@ -2494,42 +2494,42 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Tuskys Eldoret Branch</t>
+          <t>Quickmart Maua Branch</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Tuskys</t>
+          <t>Quickmart</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Express</t>
+          <t>Supermarket</t>
         </is>
       </c>
       <c r="E43" t="n">
-        <v>1285</v>
+        <v>3920</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Uasin Gishu</t>
+          <t>Meru</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Rift Valley</t>
+          <t>Eastern</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>Eldoret</t>
+          <t>Maua</t>
         </is>
       </c>
       <c r="I43" s="1" t="n">
-        <v>43375</v>
+        <v>42959</v>
       </c>
       <c r="J43" s="1" t="n">
-        <v>45820</v>
+        <v>45118</v>
       </c>
       <c r="K43" t="b">
         <v>1</v>
@@ -2543,42 +2543,42 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Carrefour Thika Branch</t>
+          <t>Eastmatt Ngong Branch</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Carrefour</t>
+          <t>Eastmatt</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Express</t>
+          <t>Supermarket</t>
         </is>
       </c>
       <c r="E44" t="n">
-        <v>1740</v>
+        <v>3733</v>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Kiambu</t>
+          <t>Kajiado</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Central</t>
+          <t>Rift Valley</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>Thika</t>
+          <t>Ngong</t>
         </is>
       </c>
       <c r="I44" s="1" t="n">
-        <v>43812</v>
+        <v>43582</v>
       </c>
       <c r="J44" s="1" t="n">
-        <v>45768</v>
+        <v>44682</v>
       </c>
       <c r="K44" t="b">
         <v>1</v>
@@ -2592,42 +2592,42 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Carrefour Maua Branch</t>
+          <t>Magunas Gilgil Branch</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Carrefour</t>
+          <t>Magunas</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Express</t>
+          <t>Supermarket</t>
         </is>
       </c>
       <c r="E45" t="n">
-        <v>1826</v>
+        <v>3542</v>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Meru</t>
+          <t>Nakuru</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Eastern</t>
+          <t>Rift Valley</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>Maua</t>
+          <t>Gilgil</t>
         </is>
       </c>
       <c r="I45" s="1" t="n">
-        <v>42838</v>
+        <v>43750</v>
       </c>
       <c r="J45" s="1" t="n">
-        <v>44611</v>
+        <v>44323</v>
       </c>
       <c r="K45" t="b">
         <v>1</v>
@@ -2641,7 +2641,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Tuskys Machakos Town Branch</t>
+          <t>Tuskys Kikuyu Branch</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2651,32 +2651,32 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Hypermarket</t>
+          <t>Supermarket</t>
         </is>
       </c>
       <c r="E46" t="n">
-        <v>8882</v>
+        <v>4405</v>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Machakos</t>
+          <t>Kiambu</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Eastern</t>
+          <t>Central</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>Machakos Town</t>
+          <t>Kikuyu</t>
         </is>
       </c>
       <c r="I46" s="1" t="n">
-        <v>42730</v>
+        <v>42628</v>
       </c>
       <c r="J46" s="1" t="n">
-        <v>45566</v>
+        <v>43997</v>
       </c>
       <c r="K46" t="b">
         <v>1</v>
@@ -2690,12 +2690,12 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Eastmatt Kitale Branch</t>
+          <t>Carrefour Mlolongo Branch</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Eastmatt</t>
+          <t>Carrefour</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -2704,28 +2704,28 @@
         </is>
       </c>
       <c r="E47" t="n">
-        <v>1746</v>
+        <v>1335</v>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Trans Nzoia</t>
+          <t>Machakos</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Rift Valley</t>
+          <t>Eastern</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>Kitale</t>
+          <t>Mlolongo</t>
         </is>
       </c>
       <c r="I47" s="1" t="n">
-        <v>42115</v>
+        <v>42308</v>
       </c>
       <c r="J47" s="1" t="n">
-        <v>44235</v>
+        <v>44205</v>
       </c>
       <c r="K47" t="b">
         <v>1</v>
@@ -2739,12 +2739,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Naivas Kilimani Branch</t>
+          <t>Carrefour Embu Town Branch</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Naivas</t>
+          <t>Carrefour</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -2753,28 +2753,28 @@
         </is>
       </c>
       <c r="E48" t="n">
-        <v>1347</v>
+        <v>1405</v>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Nairobi</t>
+          <t>Embu</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Nairobi</t>
+          <t>Eastern</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>Kilimani</t>
+          <t>Embu Town</t>
         </is>
       </c>
       <c r="I48" s="1" t="n">
-        <v>43644</v>
+        <v>43056</v>
       </c>
       <c r="J48" s="1" t="n">
-        <v>44279</v>
+        <v>44032</v>
       </c>
       <c r="K48" t="b">
         <v>1</v>
@@ -2788,12 +2788,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Carrefour Bungoma Town Branch</t>
+          <t>Chandarana Kakamega Town Branch</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Carrefour</t>
+          <t>Chandarana</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -2802,11 +2802,11 @@
         </is>
       </c>
       <c r="E49" t="n">
-        <v>4098</v>
+        <v>3356</v>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Bungoma</t>
+          <t>Kakamega</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -2816,14 +2816,14 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>Bungoma Town</t>
+          <t>Kakamega Town</t>
         </is>
       </c>
       <c r="I49" s="1" t="n">
-        <v>42923</v>
+        <v>42068</v>
       </c>
       <c r="J49" s="1" t="n">
-        <v>44406</v>
+        <v>45488</v>
       </c>
       <c r="K49" t="b">
         <v>1</v>
@@ -2837,42 +2837,42 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Eastmatt Eldoret Branch</t>
+          <t>Magunas Nairobi CBD Branch</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Eastmatt</t>
+          <t>Magunas</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Supermarket</t>
+          <t>Express</t>
         </is>
       </c>
       <c r="E50" t="n">
-        <v>3947</v>
+        <v>1563</v>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Uasin Gishu</t>
+          <t>Nairobi</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Rift Valley</t>
+          <t>Nairobi</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>Eldoret</t>
+          <t>Nairobi CBD</t>
         </is>
       </c>
       <c r="I50" s="1" t="n">
         <v>42516</v>
       </c>
       <c r="J50" s="1" t="n">
-        <v>44140</v>
+        <v>44219</v>
       </c>
       <c r="K50" t="b">
         <v>1</v>
@@ -2886,7 +2886,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Magunas Ruaka Branch</t>
+          <t>Magunas Maua Branch</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2896,32 +2896,32 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Express</t>
+          <t>Supermarket</t>
         </is>
       </c>
       <c r="E51" t="n">
-        <v>1876</v>
+        <v>4625</v>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Nairobi</t>
+          <t>Meru</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Nairobi</t>
+          <t>Eastern</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>Ruaka</t>
+          <t>Maua</t>
         </is>
       </c>
       <c r="I51" s="1" t="n">
-        <v>43132</v>
+        <v>42291</v>
       </c>
       <c r="J51" s="1" t="n">
-        <v>44233</v>
+        <v>44329</v>
       </c>
       <c r="K51" t="b">
         <v>1</v>
@@ -2935,7 +2935,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Naivas Nairobi CBD Branch</t>
+          <t>Naivas Eldoret Branch</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2945,32 +2945,32 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Express</t>
+          <t>Hypermarket</t>
         </is>
       </c>
       <c r="E52" t="n">
-        <v>1553</v>
+        <v>9599</v>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Nairobi</t>
+          <t>Uasin Gishu</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Nairobi</t>
+          <t>Rift Valley</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>Nairobi CBD</t>
+          <t>Eldoret</t>
         </is>
       </c>
       <c r="I52" s="1" t="n">
-        <v>43717</v>
+        <v>42460</v>
       </c>
       <c r="J52" s="1" t="n">
-        <v>43892</v>
+        <v>44367</v>
       </c>
       <c r="K52" t="b">
         <v>1</v>
@@ -2984,12 +2984,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Tuskys Ruiru Branch</t>
+          <t>Carrefour Eastleigh Branch</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Tuskys</t>
+          <t>Carrefour</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -2998,28 +2998,28 @@
         </is>
       </c>
       <c r="E53" t="n">
-        <v>1869</v>
+        <v>1381</v>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Kiambu</t>
+          <t>Nairobi</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Central</t>
+          <t>Nairobi</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>Ruiru</t>
+          <t>Eastleigh</t>
         </is>
       </c>
       <c r="I53" s="1" t="n">
-        <v>42489</v>
+        <v>43410</v>
       </c>
       <c r="J53" s="1" t="n">
-        <v>44513</v>
+        <v>44176</v>
       </c>
       <c r="K53" t="b">
         <v>1</v>
@@ -3033,12 +3033,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Eastmatt Nyali Branch</t>
+          <t>Chandarana Ruiru Branch</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Eastmatt</t>
+          <t>Chandarana</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -3047,28 +3047,28 @@
         </is>
       </c>
       <c r="E54" t="n">
-        <v>1218</v>
+        <v>1076</v>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Mombasa</t>
+          <t>Kiambu</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Coast</t>
+          <t>Central</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>Nyali</t>
+          <t>Ruiru</t>
         </is>
       </c>
       <c r="I54" s="1" t="n">
-        <v>43775</v>
+        <v>42049</v>
       </c>
       <c r="J54" s="1" t="n">
-        <v>45474</v>
+        <v>44096</v>
       </c>
       <c r="K54" t="b">
         <v>1</v>
@@ -3082,42 +3082,42 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Naivas Thika Branch</t>
+          <t>Carrefour Kilimani Branch</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Naivas</t>
+          <t>Carrefour</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Supermarket</t>
+          <t>Express</t>
         </is>
       </c>
       <c r="E55" t="n">
-        <v>3004</v>
+        <v>1454</v>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Kiambu</t>
+          <t>Nairobi</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Central</t>
+          <t>Nairobi</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>Thika</t>
+          <t>Kilimani</t>
         </is>
       </c>
       <c r="I55" s="1" t="n">
-        <v>42804</v>
+        <v>43662</v>
       </c>
       <c r="J55" s="1" t="n">
-        <v>44918</v>
+        <v>44359</v>
       </c>
       <c r="K55" t="b">
         <v>1</v>
@@ -3131,42 +3131,42 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Magunas Eldoret Branch</t>
+          <t>Tuskys Diani Branch</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Magunas</t>
+          <t>Tuskys</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Supermarket</t>
+          <t>Express</t>
         </is>
       </c>
       <c r="E56" t="n">
-        <v>4426</v>
+        <v>1849</v>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Uasin Gishu</t>
+          <t>Kwale</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>Rift Valley</t>
+          <t>Coast</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>Eldoret</t>
+          <t>Diani</t>
         </is>
       </c>
       <c r="I56" s="1" t="n">
-        <v>43501</v>
+        <v>43661</v>
       </c>
       <c r="J56" s="1" t="n">
-        <v>45825</v>
+        <v>45190</v>
       </c>
       <c r="K56" t="b">
         <v>1</v>
@@ -3180,42 +3180,42 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Quickmart Machakos Town Branch</t>
+          <t>Tuskys Nairobi CBD Branch</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Quickmart</t>
+          <t>Tuskys</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Supermarket</t>
+          <t>Hypermarket</t>
         </is>
       </c>
       <c r="E57" t="n">
-        <v>3445</v>
+        <v>8944</v>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Machakos</t>
+          <t>Nairobi</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>Eastern</t>
+          <t>Nairobi</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>Machakos Town</t>
+          <t>Nairobi CBD</t>
         </is>
       </c>
       <c r="I57" s="1" t="n">
-        <v>42124</v>
+        <v>42108</v>
       </c>
       <c r="J57" s="1" t="n">
-        <v>44081</v>
+        <v>44520</v>
       </c>
       <c r="K57" t="b">
         <v>1</v>
@@ -3229,42 +3229,42 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Cleanshelf Ngong Branch</t>
+          <t>Eastmatt Nairobi CBD Branch</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Cleanshelf</t>
+          <t>Eastmatt</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Hypermarket</t>
+          <t>Express</t>
         </is>
       </c>
       <c r="E58" t="n">
-        <v>9196</v>
+        <v>1404</v>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Kajiado</t>
+          <t>Nairobi</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Rift Valley</t>
+          <t>Nairobi</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>Ngong</t>
+          <t>Nairobi CBD</t>
         </is>
       </c>
       <c r="I58" s="1" t="n">
-        <v>42981</v>
+        <v>43021</v>
       </c>
       <c r="J58" s="1" t="n">
-        <v>45891</v>
+        <v>43952</v>
       </c>
       <c r="K58" t="b">
         <v>1</v>
@@ -3278,42 +3278,42 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Quickmart Meru Town Branch</t>
+          <t>Eastmatt Kilimani Branch</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Quickmart</t>
+          <t>Eastmatt</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Hypermarket</t>
+          <t>Express</t>
         </is>
       </c>
       <c r="E59" t="n">
-        <v>9040</v>
+        <v>1176</v>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Meru</t>
+          <t>Nairobi</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Eastern</t>
+          <t>Nairobi</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>Meru Town</t>
+          <t>Kilimani</t>
         </is>
       </c>
       <c r="I59" s="1" t="n">
-        <v>42169</v>
+        <v>42729</v>
       </c>
       <c r="J59" s="1" t="n">
-        <v>44593</v>
+        <v>44711</v>
       </c>
       <c r="K59" t="b">
         <v>1</v>
@@ -3327,42 +3327,42 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Tuskys Bungoma Town Branch</t>
+          <t>Quickmart Machakos Town Branch</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Tuskys</t>
+          <t>Quickmart</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Express</t>
+          <t>Supermarket</t>
         </is>
       </c>
       <c r="E60" t="n">
-        <v>1691</v>
+        <v>3913</v>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Bungoma</t>
+          <t>Machakos</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Western</t>
+          <t>Eastern</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>Bungoma Town</t>
+          <t>Machakos Town</t>
         </is>
       </c>
       <c r="I60" s="1" t="n">
-        <v>43770</v>
+        <v>43814</v>
       </c>
       <c r="J60" s="1" t="n">
-        <v>44795</v>
+        <v>44440</v>
       </c>
       <c r="K60" t="b">
         <v>1</v>
@@ -3376,42 +3376,42 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Eastmatt Ruaka Branch</t>
+          <t>Naivas Diani Branch</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Eastmatt</t>
+          <t>Naivas</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Supermarket</t>
+          <t>Express</t>
         </is>
       </c>
       <c r="E61" t="n">
-        <v>4823</v>
+        <v>1631</v>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Nairobi</t>
+          <t>Kwale</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>Nairobi</t>
+          <t>Coast</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>Ruaka</t>
+          <t>Diani</t>
         </is>
       </c>
       <c r="I61" s="1" t="n">
-        <v>43171</v>
+        <v>42508</v>
       </c>
       <c r="J61" s="1" t="n">
-        <v>44840</v>
+        <v>45040</v>
       </c>
       <c r="K61" t="b">
         <v>1</v>
@@ -3425,12 +3425,12 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Naivas Ruaka Branch</t>
+          <t>Magunas Kikuyu Branch</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Naivas</t>
+          <t>Magunas</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -3439,28 +3439,28 @@
         </is>
       </c>
       <c r="E62" t="n">
-        <v>1429</v>
+        <v>1563</v>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Nairobi</t>
+          <t>Kiambu</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>Nairobi</t>
+          <t>Central</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>Ruaka</t>
+          <t>Kikuyu</t>
         </is>
       </c>
       <c r="I62" s="1" t="n">
-        <v>43351</v>
+        <v>42986</v>
       </c>
       <c r="J62" s="1" t="n">
-        <v>45973</v>
+        <v>44081</v>
       </c>
       <c r="K62" t="b">
         <v>1</v>
@@ -3474,42 +3474,42 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Cleanshelf Nyali Branch</t>
+          <t>Tuskys Maua Branch</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Cleanshelf</t>
+          <t>Tuskys</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Express</t>
+          <t>Supermarket</t>
         </is>
       </c>
       <c r="E63" t="n">
-        <v>1209</v>
+        <v>3281</v>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Mombasa</t>
+          <t>Meru</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>Coast</t>
+          <t>Eastern</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>Nyali</t>
+          <t>Maua</t>
         </is>
       </c>
       <c r="I63" s="1" t="n">
-        <v>43376</v>
+        <v>42863</v>
       </c>
       <c r="J63" s="1" t="n">
-        <v>45118</v>
+        <v>44648</v>
       </c>
       <c r="K63" t="b">
         <v>1</v>
@@ -3523,7 +3523,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Carrefour Makutano Branch</t>
+          <t>Carrefour Meru Town Branch</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -3533,11 +3533,11 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Supermarket</t>
+          <t>Express</t>
         </is>
       </c>
       <c r="E64" t="n">
-        <v>3268</v>
+        <v>1821</v>
       </c>
       <c r="F64" t="inlineStr">
         <is>
@@ -3551,14 +3551,14 @@
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>Makutano</t>
+          <t>Meru Town</t>
         </is>
       </c>
       <c r="I64" s="1" t="n">
-        <v>43380</v>
+        <v>43118</v>
       </c>
       <c r="J64" s="1" t="n">
-        <v>45060</v>
+        <v>43911</v>
       </c>
       <c r="K64" t="b">
         <v>1</v>
@@ -3572,25 +3572,25 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Magunas Maua Branch</t>
+          <t>Eastmatt Athi River Branch</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Magunas</t>
+          <t>Eastmatt</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Supermarket</t>
+          <t>Express</t>
         </is>
       </c>
       <c r="E65" t="n">
-        <v>4539</v>
+        <v>1367</v>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Meru</t>
+          <t>Machakos</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -3600,14 +3600,14 @@
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>Maua</t>
+          <t>Athi River</t>
         </is>
       </c>
       <c r="I65" s="1" t="n">
-        <v>42153</v>
+        <v>42987</v>
       </c>
       <c r="J65" s="1" t="n">
-        <v>43870</v>
+        <v>45817</v>
       </c>
       <c r="K65" t="b">
         <v>1</v>
@@ -3621,12 +3621,12 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Magunas Kitale Branch</t>
+          <t>Cleanshelf Ngong Branch</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Magunas</t>
+          <t>Cleanshelf</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -3635,11 +3635,11 @@
         </is>
       </c>
       <c r="E66" t="n">
-        <v>1576</v>
+        <v>1514</v>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>Trans Nzoia</t>
+          <t>Kajiado</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -3649,14 +3649,14 @@
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>Kitale</t>
+          <t>Ngong</t>
         </is>
       </c>
       <c r="I66" s="1" t="n">
-        <v>42209</v>
+        <v>42663</v>
       </c>
       <c r="J66" s="1" t="n">
-        <v>44132</v>
+        <v>45422</v>
       </c>
       <c r="K66" t="b">
         <v>1</v>
@@ -3670,42 +3670,42 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Carrefour Karen Branch</t>
+          <t>Chandarana Nanyuki Branch</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Carrefour</t>
+          <t>Chandarana</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Express</t>
+          <t>Supermarket</t>
         </is>
       </c>
       <c r="E67" t="n">
-        <v>1135</v>
+        <v>3653</v>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Nairobi</t>
+          <t>Laikipia</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>Nairobi</t>
+          <t>Rift Valley</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>Karen</t>
+          <t>Nanyuki</t>
         </is>
       </c>
       <c r="I67" s="1" t="n">
-        <v>42719</v>
+        <v>43227</v>
       </c>
       <c r="J67" s="1" t="n">
-        <v>44113</v>
+        <v>44729</v>
       </c>
       <c r="K67" t="b">
         <v>1</v>
@@ -3719,42 +3719,42 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Carrefour Nanyuki Branch</t>
+          <t>Naivas Athi River Branch</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Carrefour</t>
+          <t>Naivas</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Supermarket</t>
+          <t>Express</t>
         </is>
       </c>
       <c r="E68" t="n">
-        <v>3323</v>
+        <v>1797</v>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>Laikipia</t>
+          <t>Machakos</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>Rift Valley</t>
+          <t>Eastern</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>Nanyuki</t>
+          <t>Athi River</t>
         </is>
       </c>
       <c r="I68" s="1" t="n">
-        <v>42902</v>
+        <v>42580</v>
       </c>
       <c r="J68" s="1" t="n">
-        <v>45071</v>
+        <v>44071</v>
       </c>
       <c r="K68" t="b">
         <v>1</v>
@@ -3768,12 +3768,12 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Naivas Kakamega Town Branch</t>
+          <t>Magunas Kitale Branch</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Naivas</t>
+          <t>Magunas</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -3782,28 +3782,28 @@
         </is>
       </c>
       <c r="E69" t="n">
-        <v>1567</v>
+        <v>1785</v>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Kakamega</t>
+          <t>Trans Nzoia</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>Western</t>
+          <t>Rift Valley</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>Kakamega Town</t>
+          <t>Kitale</t>
         </is>
       </c>
       <c r="I69" s="1" t="n">
-        <v>42618</v>
+        <v>43201</v>
       </c>
       <c r="J69" s="1" t="n">
-        <v>44256</v>
+        <v>44785</v>
       </c>
       <c r="K69" t="b">
         <v>1</v>
@@ -3817,7 +3817,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Quickmart Nanyuki Branch</t>
+          <t>Quickmart Mlolongo Branch</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -3831,28 +3831,28 @@
         </is>
       </c>
       <c r="E70" t="n">
-        <v>4822</v>
+        <v>4345</v>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>Laikipia</t>
+          <t>Machakos</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>Rift Valley</t>
+          <t>Eastern</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>Nanyuki</t>
+          <t>Mlolongo</t>
         </is>
       </c>
       <c r="I70" s="1" t="n">
-        <v>42224</v>
+        <v>42498</v>
       </c>
       <c r="J70" s="1" t="n">
-        <v>44468</v>
+        <v>44923</v>
       </c>
       <c r="K70" t="b">
         <v>1</v>
@@ -3866,42 +3866,42 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Chandarana Ngong Branch</t>
+          <t>Naivas Mombasa CBD Branch</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Chandarana</t>
+          <t>Naivas</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Supermarket</t>
+          <t>Express</t>
         </is>
       </c>
       <c r="E71" t="n">
-        <v>3431</v>
+        <v>1970</v>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>Kajiado</t>
+          <t>Mombasa</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>Rift Valley</t>
+          <t>Coast</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>Ngong</t>
+          <t>Mombasa CBD</t>
         </is>
       </c>
       <c r="I71" s="1" t="n">
-        <v>43474</v>
+        <v>42454</v>
       </c>
       <c r="J71" s="1" t="n">
-        <v>45236</v>
+        <v>45422</v>
       </c>
       <c r="K71" t="b">
         <v>1</v>
@@ -3915,12 +3915,12 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Carrefour Kerugoya Branch</t>
+          <t>Cleanshelf Ruaka Branch</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Carrefour</t>
+          <t>Cleanshelf</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -3929,28 +3929,28 @@
         </is>
       </c>
       <c r="E72" t="n">
-        <v>1873</v>
+        <v>1865</v>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>Kirinyaga</t>
+          <t>Nairobi</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>Central</t>
+          <t>Nairobi</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>Kerugoya</t>
+          <t>Ruaka</t>
         </is>
       </c>
       <c r="I72" s="1" t="n">
-        <v>42545</v>
+        <v>42360</v>
       </c>
       <c r="J72" s="1" t="n">
-        <v>45902</v>
+        <v>44553</v>
       </c>
       <c r="K72" t="b">
         <v>1</v>
@@ -3964,42 +3964,42 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Magunas Kilifi Town Branch</t>
+          <t>Carrefour Ruaka Branch</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Magunas</t>
+          <t>Carrefour</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Supermarket</t>
+          <t>Express</t>
         </is>
       </c>
       <c r="E73" t="n">
-        <v>4859</v>
+        <v>1825</v>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>Kilifi</t>
+          <t>Nairobi</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>Coast</t>
+          <t>Nairobi</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>Kilifi Town</t>
+          <t>Ruaka</t>
         </is>
       </c>
       <c r="I73" s="1" t="n">
-        <v>43737</v>
+        <v>43516</v>
       </c>
       <c r="J73" s="1" t="n">
-        <v>44040</v>
+        <v>45301</v>
       </c>
       <c r="K73" t="b">
         <v>1</v>
@@ -4013,12 +4013,12 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Tuskys Mombasa CBD Branch</t>
+          <t>Naivas Bungoma Town Branch</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Tuskys</t>
+          <t>Naivas</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -4027,28 +4027,28 @@
         </is>
       </c>
       <c r="E74" t="n">
-        <v>1849</v>
+        <v>1360</v>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>Mombasa</t>
+          <t>Bungoma</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>Coast</t>
+          <t>Western</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>Mombasa CBD</t>
+          <t>Bungoma Town</t>
         </is>
       </c>
       <c r="I74" s="1" t="n">
-        <v>42571</v>
+        <v>43167</v>
       </c>
       <c r="J74" s="1" t="n">
-        <v>44012</v>
+        <v>44414</v>
       </c>
       <c r="K74" t="b">
         <v>1</v>
@@ -4062,42 +4062,42 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Naivas Diani Branch</t>
+          <t>Carrefour Thika Branch</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Naivas</t>
+          <t>Carrefour</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Supermarket</t>
+          <t>Express</t>
         </is>
       </c>
       <c r="E75" t="n">
-        <v>3267</v>
+        <v>1829</v>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Kwale</t>
+          <t>Kiambu</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>Coast</t>
+          <t>Central</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>Diani</t>
+          <t>Thika</t>
         </is>
       </c>
       <c r="I75" s="1" t="n">
-        <v>43309</v>
+        <v>43810</v>
       </c>
       <c r="J75" s="1" t="n">
-        <v>44904</v>
+        <v>45848</v>
       </c>
       <c r="K75" t="b">
         <v>1</v>
@@ -4111,42 +4111,42 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Quickmart Kiambu Town Branch</t>
+          <t>Chandarana Nakuru Town Branch</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Quickmart</t>
+          <t>Chandarana</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Express</t>
+          <t>Supermarket</t>
         </is>
       </c>
       <c r="E76" t="n">
-        <v>1564</v>
+        <v>3077</v>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>Kiambu</t>
+          <t>Nakuru</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>Central</t>
+          <t>Rift Valley</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>Kiambu Town</t>
+          <t>Nakuru Town</t>
         </is>
       </c>
       <c r="I76" s="1" t="n">
-        <v>43450</v>
+        <v>42189</v>
       </c>
       <c r="J76" s="1" t="n">
-        <v>45583</v>
+        <v>44062</v>
       </c>
       <c r="K76" t="b">
         <v>1</v>
@@ -4160,42 +4160,42 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Naivas Murang'a Town Branch</t>
+          <t>Carrefour Makutano Branch</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Naivas</t>
+          <t>Carrefour</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Supermarket</t>
+          <t>Express</t>
         </is>
       </c>
       <c r="E77" t="n">
-        <v>4935</v>
+        <v>1020</v>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>Murang'a</t>
+          <t>Meru</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>Central</t>
+          <t>Eastern</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>Murang'a Town</t>
+          <t>Makutano</t>
         </is>
       </c>
       <c r="I77" s="1" t="n">
-        <v>43813</v>
+        <v>43083</v>
       </c>
       <c r="J77" s="1" t="n">
-        <v>44442</v>
+        <v>45789</v>
       </c>
       <c r="K77" t="b">
         <v>1</v>
@@ -4209,7 +4209,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Naivas Gilgil Branch</t>
+          <t>Naivas Meru Town Branch</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -4219,32 +4219,32 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Express</t>
+          <t>Supermarket</t>
         </is>
       </c>
       <c r="E78" t="n">
-        <v>1596</v>
+        <v>4257</v>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>Nakuru</t>
+          <t>Meru</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>Rift Valley</t>
+          <t>Eastern</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>Gilgil</t>
+          <t>Meru Town</t>
         </is>
       </c>
       <c r="I78" s="1" t="n">
-        <v>43136</v>
+        <v>42417</v>
       </c>
       <c r="J78" s="1" t="n">
-        <v>44438</v>
+        <v>44366</v>
       </c>
       <c r="K78" t="b">
         <v>1</v>
@@ -4258,21 +4258,21 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Eastmatt Karen Branch</t>
+          <t>Cleanshelf Nairobi CBD Branch</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Eastmatt</t>
+          <t>Cleanshelf</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Supermarket</t>
+          <t>Express</t>
         </is>
       </c>
       <c r="E79" t="n">
-        <v>3631</v>
+        <v>1940</v>
       </c>
       <c r="F79" t="inlineStr">
         <is>
@@ -4286,14 +4286,14 @@
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>Karen</t>
+          <t>Nairobi CBD</t>
         </is>
       </c>
       <c r="I79" s="1" t="n">
-        <v>42751</v>
+        <v>43648</v>
       </c>
       <c r="J79" s="1" t="n">
-        <v>43995</v>
+        <v>45157</v>
       </c>
       <c r="K79" t="b">
         <v>1</v>
@@ -4307,42 +4307,42 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Cleanshelf Eastleigh Branch</t>
+          <t>Naivas Kitengela Branch</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Cleanshelf</t>
+          <t>Naivas</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Supermarket</t>
+          <t>Hypermarket</t>
         </is>
       </c>
       <c r="E80" t="n">
-        <v>3511</v>
+        <v>9201</v>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>Nairobi</t>
+          <t>Kajiado</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>Nairobi</t>
+          <t>Rift Valley</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>Eastleigh</t>
+          <t>Kitengela</t>
         </is>
       </c>
       <c r="I80" s="1" t="n">
-        <v>43370</v>
+        <v>43448</v>
       </c>
       <c r="J80" s="1" t="n">
-        <v>44253</v>
+        <v>44412</v>
       </c>
       <c r="K80" t="b">
         <v>1</v>
@@ -4356,12 +4356,12 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Cleanshelf Thika Branch</t>
+          <t>Tuskys Thika Branch</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Cleanshelf</t>
+          <t>Tuskys</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -4370,7 +4370,7 @@
         </is>
       </c>
       <c r="E81" t="n">
-        <v>1905</v>
+        <v>1881</v>
       </c>
       <c r="F81" t="inlineStr">
         <is>
@@ -4388,10 +4388,10 @@
         </is>
       </c>
       <c r="I81" s="1" t="n">
-        <v>43796</v>
+        <v>42752</v>
       </c>
       <c r="J81" s="1" t="n">
-        <v>45496</v>
+        <v>44129</v>
       </c>
       <c r="K81" t="b">
         <v>1</v>
@@ -4405,12 +4405,12 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Quickmart Nyeri Town Branch</t>
+          <t>Cleanshelf Kikuyu Branch</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Quickmart</t>
+          <t>Cleanshelf</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -4419,11 +4419,11 @@
         </is>
       </c>
       <c r="E82" t="n">
-        <v>1242</v>
+        <v>1678</v>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>Nyeri</t>
+          <t>Kiambu</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
@@ -4433,14 +4433,14 @@
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>Nyeri Town</t>
+          <t>Kikuyu</t>
         </is>
       </c>
       <c r="I82" s="1" t="n">
-        <v>43775</v>
+        <v>42815</v>
       </c>
       <c r="J82" s="1" t="n">
-        <v>44497</v>
+        <v>44245</v>
       </c>
       <c r="K82" t="b">
         <v>1</v>
@@ -4454,42 +4454,42 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Quickmart Eldoret Branch</t>
+          <t>Cleanshelf Ruiru Branch</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Quickmart</t>
+          <t>Cleanshelf</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Express</t>
+          <t>Supermarket</t>
         </is>
       </c>
       <c r="E83" t="n">
-        <v>1025</v>
+        <v>3279</v>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>Uasin Gishu</t>
+          <t>Kiambu</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>Rift Valley</t>
+          <t>Central</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>Eldoret</t>
+          <t>Ruiru</t>
         </is>
       </c>
       <c r="I83" s="1" t="n">
-        <v>42372</v>
+        <v>42327</v>
       </c>
       <c r="J83" s="1" t="n">
-        <v>45192</v>
+        <v>45621</v>
       </c>
       <c r="K83" t="b">
         <v>1</v>
@@ -4503,12 +4503,12 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Eastmatt Diani Branch</t>
+          <t>Magunas Machakos Town Branch</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Eastmatt</t>
+          <t>Magunas</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -4517,28 +4517,28 @@
         </is>
       </c>
       <c r="E84" t="n">
-        <v>1884</v>
+        <v>1178</v>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>Kwale</t>
+          <t>Machakos</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>Coast</t>
+          <t>Eastern</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>Diani</t>
+          <t>Machakos Town</t>
         </is>
       </c>
       <c r="I84" s="1" t="n">
-        <v>43510</v>
+        <v>43453</v>
       </c>
       <c r="J84" s="1" t="n">
-        <v>44848</v>
+        <v>45293</v>
       </c>
       <c r="K84" t="b">
         <v>1</v>
@@ -4552,42 +4552,42 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Chandarana Makutano Branch</t>
+          <t>Carrefour Karen Branch</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Chandarana</t>
+          <t>Carrefour</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Supermarket</t>
+          <t>Express</t>
         </is>
       </c>
       <c r="E85" t="n">
-        <v>4436</v>
+        <v>1834</v>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>Meru</t>
+          <t>Nairobi</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>Eastern</t>
+          <t>Nairobi</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>Makutano</t>
+          <t>Karen</t>
         </is>
       </c>
       <c r="I85" s="1" t="n">
-        <v>42226</v>
+        <v>42364</v>
       </c>
       <c r="J85" s="1" t="n">
-        <v>45398</v>
+        <v>45381</v>
       </c>
       <c r="K85" t="b">
         <v>1</v>
@@ -4601,12 +4601,12 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Naivas Kitale Branch</t>
+          <t>Chandarana Eldoret Branch</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Naivas</t>
+          <t>Chandarana</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -4615,11 +4615,11 @@
         </is>
       </c>
       <c r="E86" t="n">
-        <v>1227</v>
+        <v>1301</v>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>Trans Nzoia</t>
+          <t>Uasin Gishu</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
@@ -4629,14 +4629,14 @@
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>Kitale</t>
+          <t>Eldoret</t>
         </is>
       </c>
       <c r="I86" s="1" t="n">
-        <v>42413</v>
+        <v>42265</v>
       </c>
       <c r="J86" s="1" t="n">
-        <v>45717</v>
+        <v>44559</v>
       </c>
       <c r="K86" t="b">
         <v>1</v>
@@ -4650,42 +4650,42 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Cleanshelf Kitengela Branch</t>
+          <t>Naivas Machakos Town Branch</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Cleanshelf</t>
+          <t>Naivas</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Supermarket</t>
+          <t>Express</t>
         </is>
       </c>
       <c r="E87" t="n">
-        <v>4628</v>
+        <v>1971</v>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>Kajiado</t>
+          <t>Machakos</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>Rift Valley</t>
+          <t>Eastern</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>Kitengela</t>
+          <t>Machakos Town</t>
         </is>
       </c>
       <c r="I87" s="1" t="n">
-        <v>43789</v>
+        <v>43178</v>
       </c>
       <c r="J87" s="1" t="n">
-        <v>44764</v>
+        <v>45435</v>
       </c>
       <c r="K87" t="b">
         <v>1</v>
@@ -4699,42 +4699,42 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Carrefour Machakos Town Branch</t>
+          <t>Naivas Kitale Branch</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Carrefour</t>
+          <t>Naivas</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Hypermarket</t>
+          <t>Supermarket</t>
         </is>
       </c>
       <c r="E88" t="n">
-        <v>8395</v>
+        <v>3651</v>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>Machakos</t>
+          <t>Trans Nzoia</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>Eastern</t>
+          <t>Rift Valley</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>Machakos Town</t>
+          <t>Kitale</t>
         </is>
       </c>
       <c r="I88" s="1" t="n">
-        <v>42821</v>
+        <v>43661</v>
       </c>
       <c r="J88" s="1" t="n">
-        <v>45176</v>
+        <v>44736</v>
       </c>
       <c r="K88" t="b">
         <v>1</v>
@@ -4748,12 +4748,12 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Chandarana Karen Branch</t>
+          <t>Tuskys Westlands Branch</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Chandarana</t>
+          <t>Tuskys</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -4762,7 +4762,7 @@
         </is>
       </c>
       <c r="E89" t="n">
-        <v>1990</v>
+        <v>1144</v>
       </c>
       <c r="F89" t="inlineStr">
         <is>
@@ -4776,14 +4776,14 @@
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>Karen</t>
+          <t>Westlands</t>
         </is>
       </c>
       <c r="I89" s="1" t="n">
-        <v>43588</v>
+        <v>42683</v>
       </c>
       <c r="J89" s="1" t="n">
-        <v>44975</v>
+        <v>44150</v>
       </c>
       <c r="K89" t="b">
         <v>1</v>
@@ -4797,42 +4797,42 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Cleanshelf Meru Town Branch</t>
+          <t>Carrefour Kitale Branch</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Cleanshelf</t>
+          <t>Carrefour</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Express</t>
+          <t>Supermarket</t>
         </is>
       </c>
       <c r="E90" t="n">
-        <v>1409</v>
+        <v>3654</v>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>Meru</t>
+          <t>Trans Nzoia</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>Eastern</t>
+          <t>Rift Valley</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>Meru Town</t>
+          <t>Kitale</t>
         </is>
       </c>
       <c r="I90" s="1" t="n">
-        <v>43396</v>
+        <v>42348</v>
       </c>
       <c r="J90" s="1" t="n">
-        <v>45188</v>
+        <v>44195</v>
       </c>
       <c r="K90" t="b">
         <v>1</v>
@@ -4846,42 +4846,42 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Naivas Athi River Branch</t>
+          <t>Cleanshelf Karen Branch</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Naivas</t>
+          <t>Cleanshelf</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Supermarket</t>
+          <t>Express</t>
         </is>
       </c>
       <c r="E91" t="n">
-        <v>4987</v>
+        <v>1271</v>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>Machakos</t>
+          <t>Nairobi</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>Eastern</t>
+          <t>Nairobi</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>Athi River</t>
+          <t>Karen</t>
         </is>
       </c>
       <c r="I91" s="1" t="n">
-        <v>42539</v>
+        <v>42434</v>
       </c>
       <c r="J91" s="1" t="n">
-        <v>44563</v>
+        <v>44854</v>
       </c>
       <c r="K91" t="b">
         <v>1</v>
@@ -4895,42 +4895,42 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Chandarana Eastleigh Branch</t>
+          <t>Tuskys Machakos Town Branch</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Chandarana</t>
+          <t>Tuskys</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Hypermarket</t>
+          <t>Supermarket</t>
         </is>
       </c>
       <c r="E92" t="n">
-        <v>9221</v>
+        <v>4611</v>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>Nairobi</t>
+          <t>Machakos</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>Nairobi</t>
+          <t>Eastern</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>Eastleigh</t>
+          <t>Machakos Town</t>
         </is>
       </c>
       <c r="I92" s="1" t="n">
-        <v>42894</v>
+        <v>42226</v>
       </c>
       <c r="J92" s="1" t="n">
-        <v>45247</v>
+        <v>43837</v>
       </c>
       <c r="K92" t="b">
         <v>1</v>
@@ -4944,42 +4944,42 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Cleanshelf Mlolongo Branch</t>
+          <t>Naivas Westlands Branch</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Cleanshelf</t>
+          <t>Naivas</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Express</t>
+          <t>Supermarket</t>
         </is>
       </c>
       <c r="E93" t="n">
-        <v>1523</v>
+        <v>4500</v>
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>Machakos</t>
+          <t>Nairobi</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>Eastern</t>
+          <t>Nairobi</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>Mlolongo</t>
+          <t>Westlands</t>
         </is>
       </c>
       <c r="I93" s="1" t="n">
-        <v>42241</v>
+        <v>42864</v>
       </c>
       <c r="J93" s="1" t="n">
-        <v>45409</v>
+        <v>44513</v>
       </c>
       <c r="K93" t="b">
         <v>1</v>
@@ -4993,42 +4993,42 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Carrefour Naivasha Branch</t>
+          <t>Eastmatt Murang'a Town Branch</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Carrefour</t>
+          <t>Eastmatt</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Supermarket</t>
+          <t>Express</t>
         </is>
       </c>
       <c r="E94" t="n">
-        <v>4451</v>
+        <v>1387</v>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>Nakuru</t>
+          <t>Murang'a</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>Rift Valley</t>
+          <t>Central</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>Naivasha</t>
+          <t>Murang'a Town</t>
         </is>
       </c>
       <c r="I94" s="1" t="n">
-        <v>42898</v>
+        <v>42724</v>
       </c>
       <c r="J94" s="1" t="n">
-        <v>43838</v>
+        <v>45369</v>
       </c>
       <c r="K94" t="b">
         <v>1</v>
@@ -5042,42 +5042,42 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Carrefour Eastleigh Branch</t>
+          <t>Tuskys Kerugoya Branch</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Carrefour</t>
+          <t>Tuskys</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Supermarket</t>
+          <t>Express</t>
         </is>
       </c>
       <c r="E95" t="n">
-        <v>3143</v>
+        <v>1807</v>
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>Nairobi</t>
+          <t>Kirinyaga</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>Nairobi</t>
+          <t>Central</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>Eastleigh</t>
+          <t>Kerugoya</t>
         </is>
       </c>
       <c r="I95" s="1" t="n">
-        <v>43365</v>
+        <v>43774</v>
       </c>
       <c r="J95" s="1" t="n">
-        <v>45184</v>
+        <v>44755</v>
       </c>
       <c r="K95" t="b">
         <v>1</v>
@@ -5091,12 +5091,12 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Cleanshelf Makutano Branch</t>
+          <t>Quickmart Eastleigh Branch</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Cleanshelf</t>
+          <t>Quickmart</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -5105,28 +5105,28 @@
         </is>
       </c>
       <c r="E96" t="n">
-        <v>1127</v>
+        <v>1818</v>
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>Meru</t>
+          <t>Nairobi</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>Eastern</t>
+          <t>Nairobi</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>Makutano</t>
+          <t>Eastleigh</t>
         </is>
       </c>
       <c r="I96" s="1" t="n">
-        <v>43479</v>
+        <v>43737</v>
       </c>
       <c r="J96" s="1" t="n">
-        <v>45062</v>
+        <v>43968</v>
       </c>
       <c r="K96" t="b">
         <v>1</v>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Chandarana Embu Town Branch</t>
+          <t>Chandarana Kikuyu Branch</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -5150,32 +5150,32 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Express</t>
+          <t>Hypermarket</t>
         </is>
       </c>
       <c r="E97" t="n">
-        <v>1334</v>
+        <v>8534</v>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>Embu</t>
+          <t>Kiambu</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>Eastern</t>
+          <t>Central</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>Embu Town</t>
+          <t>Kikuyu</t>
         </is>
       </c>
       <c r="I97" s="1" t="n">
-        <v>42829</v>
+        <v>42219</v>
       </c>
       <c r="J97" s="1" t="n">
-        <v>45043</v>
+        <v>44135</v>
       </c>
       <c r="K97" t="b">
         <v>1</v>
@@ -5189,12 +5189,12 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Quickmart Kitengela Branch</t>
+          <t>Cleanshelf Gilgil Branch</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Quickmart</t>
+          <t>Cleanshelf</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -5203,11 +5203,11 @@
         </is>
       </c>
       <c r="E98" t="n">
-        <v>4361</v>
+        <v>3768</v>
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>Kajiado</t>
+          <t>Nakuru</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
@@ -5217,14 +5217,14 @@
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>Kitengela</t>
+          <t>Gilgil</t>
         </is>
       </c>
       <c r="I98" s="1" t="n">
-        <v>42781</v>
+        <v>42334</v>
       </c>
       <c r="J98" s="1" t="n">
-        <v>44544</v>
+        <v>44139</v>
       </c>
       <c r="K98" t="b">
         <v>1</v>
@@ -5238,25 +5238,25 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Chandarana Kitale Branch</t>
+          <t>Tuskys Eldoret Branch</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Chandarana</t>
+          <t>Tuskys</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Express</t>
+          <t>Supermarket</t>
         </is>
       </c>
       <c r="E99" t="n">
-        <v>1853</v>
+        <v>4256</v>
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>Trans Nzoia</t>
+          <t>Uasin Gishu</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
@@ -5266,14 +5266,14 @@
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>Kitale</t>
+          <t>Eldoret</t>
         </is>
       </c>
       <c r="I99" s="1" t="n">
-        <v>42005</v>
+        <v>42993</v>
       </c>
       <c r="J99" s="1" t="n">
-        <v>45076</v>
+        <v>43958</v>
       </c>
       <c r="K99" t="b">
         <v>1</v>
@@ -5287,42 +5287,42 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Chandarana Kerugoya Branch</t>
+          <t>Eastmatt Karen Branch</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Chandarana</t>
+          <t>Eastmatt</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Supermarket</t>
+          <t>Express</t>
         </is>
       </c>
       <c r="E100" t="n">
-        <v>4609</v>
+        <v>1168</v>
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>Kirinyaga</t>
+          <t>Nairobi</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>Central</t>
+          <t>Nairobi</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>Kerugoya</t>
+          <t>Karen</t>
         </is>
       </c>
       <c r="I100" s="1" t="n">
-        <v>43192</v>
+        <v>43248</v>
       </c>
       <c r="J100" s="1" t="n">
-        <v>45151</v>
+        <v>45610</v>
       </c>
       <c r="K100" t="b">
         <v>1</v>
@@ -5336,42 +5336,42 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Magunas Kerugoya Branch</t>
+          <t>Quickmart Mombasa CBD Branch</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Magunas</t>
+          <t>Quickmart</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Express</t>
+          <t>Hypermarket</t>
         </is>
       </c>
       <c r="E101" t="n">
-        <v>1691</v>
+        <v>8678</v>
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>Kirinyaga</t>
+          <t>Mombasa</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>Central</t>
+          <t>Coast</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>Kerugoya</t>
+          <t>Mombasa CBD</t>
         </is>
       </c>
       <c r="I101" s="1" t="n">
-        <v>42442</v>
+        <v>42425</v>
       </c>
       <c r="J101" s="1" t="n">
-        <v>45925</v>
+        <v>44610</v>
       </c>
       <c r="K101" t="b">
         <v>1</v>

</xml_diff>